<commit_message>
Add per-agent chart (target vs forecast) to targets workbook
New 'גרף לפי סוכן' sheet with a horizontal bar chart comparing each
agent's target to their end-of-period forecast.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012muJ61YJv31ajNb5BHvc8B
</commit_message>
<xml_diff>
--- a/יעדי_סוכנים_אוגוסט.xlsx
+++ b/יעדי_סוכנים_אוגוסט.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet name="תוכנית יעדים אוגוסט" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="תחזית עמידה ביעד" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יעדים לפי סוכן" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="פירוט לפי סוכן ופריט" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="גרף לפי סוכן" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="יעדים לפי סוכן" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="פירוט לפי סוכן ופריט" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -278,6 +279,133 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>יעד מול תחזית לפי סוכן</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'תחזית עמידה ביעד'!C5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="1F4E78"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'תחזית עמידה ביעד'!$A$6:$A$28</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'תחזית עמידה ביעד'!$C$6:$C$28</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'תחזית עמידה ביעד'!F5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="ED7D31"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'תחזית עמידה ביעד'!$A$6:$A$28</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'תחזית עמידה ביעד'!$F$6:$F$28</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>₪</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
@@ -321,6 +449,33 @@
     </comment>
   </commentList>
 </comments>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8640000" cy="6480000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2216,6 +2371,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>עמידה ביעד לפי סוכן – יעד מול תחזית סוף תקופה (₪)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2901,7 +3078,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>